<commit_message>
QAQC STEEP N2O samples
</commit_message>
<xml_diff>
--- a/NCycle_Expt_N2O/N2O Data/Raw Data/Excel/20260505_STEEP_GCReW.xlsx
+++ b/NCycle_Expt_N2O/N2O Data/Raw Data/Excel/20260505_STEEP_GCReW.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\GlobalChangeEco\Porewater_R scripts &amp; Data\Data\Shimadzu GC\STEEP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sinet-my.sharepoint.com/personal/giessnerm_si_edu/Documents/Documents/GitHub/TAI_NCycle/NCycle_Expt_N2O/N2O Data/Raw Data/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A598E9CF-0872-4A14-A130-28D06E98D809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{A598E9CF-0872-4A14-A130-28D06E98D809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5CCFFEC6-D19C-4EF6-9C58-F0597CA3D179}"/>
   <bookViews>
-    <workbookView xWindow="1935" yWindow="2730" windowWidth="19410" windowHeight="11295" xr2:uid="{BD91B5F2-2EE8-4BB9-9259-82C885726BB3}"/>
+    <workbookView xWindow="960" yWindow="225" windowWidth="17805" windowHeight="14565" xr2:uid="{BD91B5F2-2EE8-4BB9-9259-82C885726BB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>